<commit_message>
Add path-stage renewal rules for C04 and C06.
Document C01+C02 to C04 and C01+C05 to C06 renewal discounts and gifts in the promo KB, Streamlit quick questions, and readme.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/资料库/报班活动-限时优惠与续报福利说明.xlsx
+++ b/资料库/报班活动-限时优惠与续报福利说明.xlsx
@@ -12,8 +12,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="限时优惠规则" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="续报赠课三门" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="打包报名费用" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="费用参考" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="顾问话术" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="路径阶段续报" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="费用参考" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="顾问话术" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +57,11 @@
       <name val="微软雅黑"/>
       <color rgb="005C574F"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="3">
@@ -97,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -123,6 +129,7 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -502,14 +509,13 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="68" customHeight="1">
+    <row r="2" ht="80" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>两套政策并行：限时优惠活动期间报班享学费折扣（可折上折）；只要续报进阶，即赠送三门配套课程（原理课、录播课、大赛样例课）。另：零基础一次性报「入门+任意一门进阶」或一次性报整条路径A/B，同样享受折上折，并赠送三门课。折扣管学费，赠课跟续报/打包报名走。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>两套政策并行：限时优惠活动期间报班享学费折扣（可折上折）；只要续报进阶，即赠送三门配套课程（原理课、录播课、大赛样例课）。另：零基础一次性报「入门+任意一门进阶」或一次性报整条路径A/B，同样享受折上折，并赠送三门课。折扣管学费，赠课跟续报/打包报名走。另明确路径阶段续报：学完 C01+C02 后续报 C04，或学完 C01+C05 后续报 C06，同样享受续报 8 折（限时活动期间可折上折约 6.8 折），并送三门课。</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -843,7 +849,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1026,6 +1032,40 @@
       <c r="C12" s="5" t="inlineStr">
         <is>
           <t>一次性报 C01+C05+C06（大模型/Agent路径）；整单折上折，并送三门课</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>路径A阶段续报：C01+C02已学 → 续报C04</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>8折 / 限时可约6.8折</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>已完成 Python入门班与 Python数据分析班后，续报机器学习项目班；享受续报 8 折；若在限时优惠活动期间续报，可折上折约 6.8 折，并送三门课</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>路径B阶段续报：C01+C05已学 → 续报C06</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>8折 / 限时可约6.8折</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>已完成 Python入门班与 大模型应用开发班后，续报 AI智能体实战班；享受续报 8 折；若在限时优惠活动期间续报，可折上折约 6.8 折，并送三门课</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1110,7 +1150,7 @@
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>触发：正式续报任一进阶正课（C02/C05/C04/C06）即送，不要求必须在限时优惠活动期间。与限时学费折扣相互独立：限时活动期间续报可折上折，同时仍送三门课。 另：零基础一次性打包（入门+进阶 / 路径A / 路径B）同样送三门课。</t>
+          <t>触发：正式续报任一进阶正课（C02/C05/C04/C06）即送，不要求必须在限时优惠活动期间。与限时学费折扣相互独立：限时活动期间续报可折上折，同时仍送三门课。 另：零基础一次性打包（入门+进阶 / 路径A / 路径B）同样送三门课。 另：路径阶段续报（C01+C02→C04；C01+C05→C06）同样送三门课。</t>
         </is>
       </c>
     </row>
@@ -1123,6 +1163,18 @@
       <c r="B9" s="5" t="inlineStr">
         <is>
           <t>零基础一次性报「C01+任意一门进阶」或整条路径A/B，与续报相同：赠送原理课、录播课、大赛样例课三门；报名确认后由教务一并开通。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>路径阶段续报同样送</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>学完 C01+C02 后续报 C04，或学完 C01+C05 后续报 C06：与普通续报相同，赠送原理课、录播课、大赛样例课三门。</t>
         </is>
       </c>
     </row>
@@ -1389,6 +1441,138 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>路径阶段续报说明（学完衔接课后再续实战课）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>适用学员已完成对应先修组合。续报实战课享受：续报 8 折；限时优惠活动期间续报可折上折约 6.8 折；并送三门课（原理课/录播课/大赛样例课）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>路径</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>已学组合</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>续报课程</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>原价（元）</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>续报8折</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>折上折约6.8折</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>路径A：数据/传统建模</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>C01 Python入门班 + C02 Python数据分析班</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>C04 机器学习项目班</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>6980</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>5584</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>4746</v>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>路径B：大模型/Agent</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>C01 Python入门班 + C05 大模型应用开发班</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>C06 AI智能体实战班</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>7580</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>6064</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>5154</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>赠课：上述两种路径阶段续报均送三门课。最终以报名系统/顾问报价单为准。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1407,6 +1591,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
@@ -1535,7 +1720,7 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>送三门</t>
+          <t>送三门（含路径A：C01+C02后续报）</t>
         </is>
       </c>
     </row>
@@ -1559,14 +1744,15 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>送三门</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>说明：金额四舍五入到元，最终以报名系统/顾问报价单为准。C01无续报8折与续报赠课。</t>
+          <t>送三门（含路径B：C01+C05后续报）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>说明：金额四舍五入到元，最终以报名系统/顾问报价单为准。C01无续报8折与续报赠课。 路径阶段续报：已学完 C01+C02 后续报 C04，或已学完 C01+C05 后续报 C06，按该课「仅续报8折 / 折上折约6.8折」列计价，并送三门。</t>
         </is>
       </c>
     </row>
@@ -1579,13 +1765,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1661,32 +1847,56 @@
       </c>
     </row>
     <row r="8"/>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>内部培训/对外咨询参考稿 · 与「课程路径-基础与进阶」配套使用 · 最终解释权归教培机构</t>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>路径A阶段续报</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>您已学完入门班和数据分析班，下一步续报机器学习项目班可以走续报 8 折；赶上限时活动还能折上折大约 6.8 折，并且送三门配套课。</t>
         </is>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>路径B阶段续报</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>您已学完入门班和大模型应用开发班，续报 AI智能体实战班同样续报 8 折；限时活动期间可折上折约 6.8 折，并送原理课、录播课、大赛样例课。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>内部培训/对外咨询参考稿 · 与「课程路径-基础与进阶」配套使用 · 最终解释权归教培机构</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
           <t>零基础一次性打包（入门+进阶）</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>零基础可以一次报入门班加任意一门进阶，整单按折上折大约6.8折算，并且送原理课、录播课、大赛样例课三门。</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="44" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>零基础一次性报路径A/B</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>如果目标明确，也可以一次报整条路径：路径A是入门+数据分析+机器学习，路径B是入门+大模型+智能体；同样折上折并送三门课。</t>
         </is>

</xml_diff>